<commit_message>
Adicinado casos de testes
</commit_message>
<xml_diff>
--- a/relatorio/Relatorio_de_Testes_CineLume.xlsx
+++ b/relatorio/Relatorio_de_Testes_CineLume.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aluno\Pictures\curso_ds\testes\git\cinelume-qa\relatorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1E95289-4E0E-4943-A134-54884266A429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0F8592E-632E-4C44-A854-2013A6EAE24A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0_Instrucoes" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="552">
   <si>
     <t>Relatório de Testes — CineLume v1.0</t>
   </si>
@@ -1562,42 +1562,9 @@
     <t>Todos elemento de ui funcionando corretamente.</t>
   </si>
   <si>
-    <t>Cupom Pipoca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">o requisito diz que um ingresso + pipoca grande o desconto é de R$ 3,20 </t>
-  </si>
-  <si>
-    <t>Alguma messagem que explique que o desconto é somente para o valor do ingresso</t>
-  </si>
-  <si>
-    <t>Desconto Pix</t>
-  </si>
-  <si>
-    <t>Alterna entre o pagamento pix e cartão acumula desconto do pix</t>
-  </si>
-  <si>
-    <t>O desconto do pix não pode ser acumulativo</t>
-  </si>
-  <si>
-    <t>Parcelamento do Cartao</t>
-  </si>
-  <si>
-    <t>limiites de centavos não permite o parcelamento para 6x</t>
-  </si>
-  <si>
-    <t>porque não colocar o valor minimo baseado no consumo medio?</t>
-  </si>
-  <si>
     <t>Nome Completo</t>
   </si>
   <si>
-    <t xml:space="preserve">Não exite nome com no minido 3 caracteres </t>
-  </si>
-  <si>
-    <t>Colocar nome completo separado por espacos</t>
-  </si>
-  <si>
     <t xml:space="preserve">Selecao de filmes,  Selecao de acentos, adicinar item na bomboniere, escolher forma de pagamento , Dados pessoais </t>
   </si>
   <si>
@@ -1631,35 +1598,125 @@
     <t>verificar se todas as funciononalidade do sistema estão de acordo com os requisitos de negocio</t>
   </si>
   <si>
-    <t>CA01.2</t>
-  </si>
-  <si>
-    <t>Preco por Horario</t>
-  </si>
-  <si>
-    <t>Acento não selecionado</t>
-  </si>
-  <si>
-    <t>1.Selecionar horario, 2.Selecionar Acento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor do ingresso R$32,00 </t>
-  </si>
-  <si>
-    <t>Preco por Horario antes das cinco</t>
-  </si>
-  <si>
-    <t>1. Selecionar horario antes das cinco                 2. Selecionar Acento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor do ingresso R$24,00 </t>
+    <t xml:space="preserve">Desconto pix </t>
+  </si>
+  <si>
+    <t>O requisito define um limite que não faz sentido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Definir um novo limite baseado na soma dos vendidos </t>
+  </si>
+  <si>
+    <t>a quantidade de caracteres para um nome e muito pequena baseado no padrao de nome brasileiro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exite algum nome com 3 caracteres?. </t>
+  </si>
+  <si>
+    <t>Com as correções verificar se o sistema esta funcinando corretamente</t>
+  </si>
+  <si>
+    <t>Tenta identificar erros que não tenha no plano de teste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simular se sistema aguenta uma quantidade de usuario e uma pre-estreia </t>
+  </si>
+  <si>
+    <t>Para discobri quando sistema trava para tomar medidas.</t>
+  </si>
+  <si>
+    <t>Analisar quanto tempo um usuario leva pra compra um ingresso e se atividade e facil de ser exeutada</t>
+  </si>
+  <si>
+    <t>Verificar se o sistema esta de acordo com os requisitos</t>
+  </si>
+  <si>
+    <t>CA02.1</t>
+  </si>
+  <si>
+    <t>CA03.1</t>
+  </si>
+  <si>
+    <t>CA04.1</t>
+  </si>
+  <si>
+    <t>CA05.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preco da seção </t>
+  </si>
+  <si>
+    <t>acento selecionado</t>
+  </si>
+  <si>
+    <t>O valor do ingresso e exibido R$24,00</t>
+  </si>
+  <si>
+    <t>Valor da sala 3D</t>
+  </si>
+  <si>
+    <t>Horario e Acento selecionado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Selecionar Horario                                         2.Selecionar Acento                                         </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Selecionar horario com filme 3D depois das 17                                                                 2. Selecionar acento </t>
+  </si>
+  <si>
+    <t>O valor da seção tem que ser R$38,00</t>
+  </si>
+  <si>
+    <t>Aplicação de Meia entrada</t>
+  </si>
+  <si>
+    <t>1.Selecionar Horario depois da 17                      2.Selecionar acento                                          3.adicionar uma meia entrada</t>
+  </si>
+  <si>
+    <t>Digita 1 na  meia entrada</t>
+  </si>
+  <si>
+    <t>No resumo exibir o valor do ingresso com metade do preco</t>
+  </si>
+  <si>
+    <t>Pre-estreia sem meia  entrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Selecionar horario com pre-estreia                  2.selecionar acento                                           3.adicionar meia entrada </t>
+  </si>
+  <si>
+    <t>O valor do ingresso com a meia-entradada não aplicado</t>
+  </si>
+  <si>
+    <t>Não confirmar pedido sem ingresso</t>
+  </si>
+  <si>
+    <t>Selecionar horario</t>
+  </si>
+  <si>
+    <t>1.selecionar horario                                          2.confirmar pedido</t>
+  </si>
+  <si>
+    <t>Mensagem dizendo que precisa selecionar um acento para confirmar</t>
+  </si>
+  <si>
+    <t>CA05.2</t>
+  </si>
+  <si>
+    <t>Limite de acentos</t>
+  </si>
+  <si>
+    <t>1.selecionar horario                                           2.selecionar mais de 6 acentos</t>
+  </si>
+  <si>
+    <t>No resumo exibir o valor total do ingresso de acordo com 6  acentos</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1731,6 +1788,14 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1805,7 +1870,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -1858,6 +1923,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2895,7 +2963,7 @@
       </c>
       <c r="B5" s="18">
         <f>COUNTA('5_Casos_de_Teste'!G6:G45)</f>
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -4082,24 +4150,24 @@
         <v>98</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>99</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>502</v>
+        <v>514</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>460</v>
+        <v>468</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>503</v>
+        <v>515</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>504</v>
+        <v>516</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
@@ -4107,60 +4175,40 @@
         <v>100</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>484</v>
+        <v>94</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>460</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>506</v>
+        <v>517</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>486</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>508</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>460</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>509</v>
-      </c>
-      <c r="F8" s="23" t="s">
-        <v>510</v>
-      </c>
+      <c r="B8" s="8"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>511</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>460</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>512</v>
-      </c>
-      <c r="F9" s="23" t="s">
-        <v>513</v>
-      </c>
+      <c r="B9" s="8"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
@@ -4231,7 +4279,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -4261,7 +4309,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -4284,7 +4332,7 @@
         <v>111</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>524</v>
+        <v>513</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -4292,7 +4340,7 @@
         <v>112</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>514</v>
+        <v>503</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>113</v>
@@ -4303,7 +4351,7 @@
         <v>114</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>521</v>
+        <v>510</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -4322,7 +4370,7 @@
         <v>117</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>515</v>
+        <v>504</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -4330,7 +4378,7 @@
         <v>118</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>516</v>
+        <v>505</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>119</v>
@@ -4341,7 +4389,7 @@
         <v>120</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>520</v>
+        <v>509</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>121</v>
@@ -4352,7 +4400,7 @@
         <v>122</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>517</v>
+        <v>506</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>123</v>
@@ -4363,7 +4411,7 @@
         <v>124</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>518</v>
+        <v>507</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>125</v>
@@ -4374,7 +4422,7 @@
         <v>126</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>519</v>
+        <v>508</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>127</v>
@@ -4413,7 +4461,7 @@
         <v>435</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>522</v>
+        <v>511</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -4423,7 +4471,9 @@
       <c r="B20" s="8" t="s">
         <v>435</v>
       </c>
-      <c r="C20" s="8"/>
+      <c r="C20" s="23" t="s">
+        <v>519</v>
+      </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="12" t="s">
@@ -4441,7 +4491,9 @@
       <c r="B22" s="8" t="s">
         <v>435</v>
       </c>
-      <c r="C22" s="8"/>
+      <c r="C22" s="23" t="s">
+        <v>520</v>
+      </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
@@ -4452,14 +4504,16 @@
       </c>
       <c r="C23" s="8"/>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A24" s="12" t="s">
         <v>139</v>
       </c>
       <c r="B24" s="8" t="s">
         <v>435</v>
       </c>
-      <c r="C24" s="8"/>
+      <c r="C24" s="23" t="s">
+        <v>521</v>
+      </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
@@ -4468,7 +4522,9 @@
       <c r="B25" s="8" t="s">
         <v>435</v>
       </c>
-      <c r="C25" s="8"/>
+      <c r="C25" s="23" t="s">
+        <v>522</v>
+      </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
@@ -4497,14 +4553,16 @@
       </c>
       <c r="C28" s="8"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A29" s="12" t="s">
         <v>144</v>
       </c>
       <c r="B29" s="23" t="s">
         <v>435</v>
       </c>
-      <c r="C29" s="8"/>
+      <c r="C29" s="23" t="s">
+        <v>523</v>
+      </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="12" t="s">
@@ -4513,7 +4571,12 @@
       <c r="B30" s="8" t="s">
         <v>435</v>
       </c>
-      <c r="C30" s="8"/>
+      <c r="C30" s="23" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C34" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4601,7 +4664,7 @@
       <c r="H4" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="I4" s="27" t="s">
         <v>153</v>
       </c>
       <c r="J4" s="10" t="s">
@@ -4666,7 +4729,7 @@
       <c r="N5" s="14"/>
       <c r="O5" s="14"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>171</v>
       </c>
@@ -4674,135 +4737,219 @@
         <v>433</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>525</v>
-      </c>
-      <c r="D6" s="8"/>
+        <v>512</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>463</v>
+      </c>
       <c r="E6" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="F6" s="8"/>
+      <c r="F6" s="8" t="s">
+        <v>445</v>
+      </c>
       <c r="G6" s="23" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="J6" s="8"/>
       <c r="K6" s="23" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="L6" s="8"/>
       <c r="M6" s="8"/>
       <c r="N6" s="8"/>
       <c r="O6" s="8"/>
     </row>
-    <row r="7" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>172</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>433</v>
+        <v>443</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>523</v>
-      </c>
-      <c r="D7" s="8"/>
+        <v>525</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>463</v>
+      </c>
       <c r="E7" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="F7" s="8"/>
+      <c r="F7" s="8" t="s">
+        <v>445</v>
+      </c>
       <c r="G7" s="23" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="J7" s="8"/>
       <c r="K7" s="23" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
       <c r="O7" s="8"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
+      <c r="B8" s="8" t="s">
+        <v>454</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>526</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>463</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>537</v>
+      </c>
+      <c r="H8" s="23" t="s">
+        <v>533</v>
+      </c>
+      <c r="I8" s="23" t="s">
+        <v>538</v>
+      </c>
+      <c r="J8" s="23" t="s">
+        <v>539</v>
+      </c>
+      <c r="K8" s="23" t="s">
+        <v>540</v>
+      </c>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="8"/>
       <c r="O8" s="8"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
+      <c r="B9" s="8" t="s">
+        <v>462</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>527</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="G9" s="23" t="s">
+        <v>541</v>
+      </c>
+      <c r="H9" s="23" t="s">
+        <v>533</v>
+      </c>
+      <c r="I9" s="23" t="s">
+        <v>542</v>
+      </c>
+      <c r="J9" s="23" t="s">
+        <v>539</v>
+      </c>
+      <c r="K9" s="22" t="s">
+        <v>543</v>
+      </c>
       <c r="L9" s="8"/>
       <c r="M9" s="8"/>
       <c r="N9" s="8"/>
       <c r="O9" s="8"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
+      <c r="B10" s="8" t="s">
+        <v>469</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>528</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="G10" s="23" t="s">
+        <v>544</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>545</v>
+      </c>
+      <c r="I10" s="23" t="s">
+        <v>546</v>
+      </c>
       <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
+      <c r="K10" s="23" t="s">
+        <v>547</v>
+      </c>
       <c r="L10" s="8"/>
       <c r="M10" s="8"/>
       <c r="N10" s="8"/>
       <c r="O10" s="8"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
+      <c r="B11" s="8" t="s">
+        <v>469</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>548</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="G11" s="23" t="s">
+        <v>549</v>
+      </c>
+      <c r="H11" s="23" t="s">
+        <v>545</v>
+      </c>
+      <c r="I11" s="23" t="s">
+        <v>550</v>
+      </c>
       <c r="J11" s="8"/>
-      <c r="K11" s="8"/>
+      <c r="K11" s="23" t="s">
+        <v>551</v>
+      </c>
       <c r="L11" s="8"/>
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
@@ -4840,7 +4987,7 @@
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
+      <c r="K13" s="22"/>
       <c r="L13" s="8"/>
       <c r="M13" s="8"/>
       <c r="N13" s="8"/>

</xml_diff>

<commit_message>
docs: plano e casos de teste
</commit_message>
<xml_diff>
--- a/relatorio/Relatorio_de_Testes_CineLume.xlsx
+++ b/relatorio/Relatorio_de_Testes_CineLume.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aluno\Pictures\curso_ds\testes\git\cinelume-qa\relatorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBF1C50E-35CA-433D-92D0-57AF92B2D28F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{677E5D5E-C84E-4A1F-B919-AC659DBB0DCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="642">
   <si>
     <t>Relatório de Testes — CineLume v1.0</t>
   </si>
@@ -1631,128 +1631,362 @@
     <t>Verificar se o sistema esta de acordo com os requisitos</t>
   </si>
   <si>
-    <t>CA02.1</t>
-  </si>
-  <si>
-    <t>CA03.1</t>
-  </si>
-  <si>
     <t>CA04.1</t>
   </si>
   <si>
-    <t>CA05.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preco da seção </t>
-  </si>
-  <si>
-    <t>acento selecionado</t>
-  </si>
-  <si>
-    <t>O valor do ingresso e exibido R$24,00</t>
-  </si>
-  <si>
-    <t>Valor da sala 3D</t>
-  </si>
-  <si>
-    <t>Horario e Acento selecionado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Selecionar Horario                                         2.Selecionar Acento                                         </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Selecionar horario com filme 3D depois das 17                                                                 2. Selecionar acento </t>
-  </si>
-  <si>
-    <t>O valor da seção tem que ser R$38,00</t>
-  </si>
-  <si>
-    <t>Aplicação de Meia entrada</t>
-  </si>
-  <si>
-    <t>1.Selecionar Horario depois da 17                      2.Selecionar acento                                          3.adicionar uma meia entrada</t>
-  </si>
-  <si>
-    <t>Digita 1 na  meia entrada</t>
-  </si>
-  <si>
-    <t>No resumo exibir o valor do ingresso com metade do preco</t>
-  </si>
-  <si>
-    <t>Pre-estreia sem meia  entrada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Selecionar horario com pre-estreia                  2.selecionar acento                                           3.adicionar meia entrada </t>
-  </si>
-  <si>
-    <t>O valor do ingresso com a meia-entradada não aplicado</t>
-  </si>
-  <si>
-    <t>Não confirmar pedido sem ingresso</t>
-  </si>
-  <si>
-    <t>Selecionar horario</t>
-  </si>
-  <si>
-    <t>1.selecionar horario                                          2.confirmar pedido</t>
-  </si>
-  <si>
-    <t>Mensagem dizendo que precisa selecionar um acento para confirmar</t>
-  </si>
-  <si>
-    <t>CA05.2</t>
-  </si>
-  <si>
-    <t>Limite de acentos</t>
-  </si>
-  <si>
-    <t>1.selecionar horario                                           2.selecionar mais de 6 acentos</t>
-  </si>
-  <si>
-    <t>No resumo exibir o valor total do ingresso de acordo com 6  acentos</t>
-  </si>
-  <si>
     <t>CA05.3</t>
   </si>
   <si>
-    <t>Limite de acentos utrapassados</t>
-  </si>
-  <si>
-    <t>1.Selecionar horario                                          2.selecionar mais de 6 acentos</t>
-  </si>
-  <si>
-    <t>Aviso do sistema que o limite foi utrapassado</t>
-  </si>
-  <si>
     <t>CA07.1</t>
   </si>
   <si>
-    <t>Limite na bomboniere</t>
-  </si>
-  <si>
-    <t>Selecionar horario e acento</t>
-  </si>
-  <si>
-    <t>1.selecionar horario                                          2.selecionar acento                                           3.colocar na bomboniere valor acima de 10</t>
-  </si>
-  <si>
-    <t>Valor e resetado para 10</t>
-  </si>
-  <si>
-    <t>CA07.2</t>
-  </si>
-  <si>
-    <t>Numeros negativos</t>
-  </si>
-  <si>
-    <t>1. Selecionar horario                                         2. Selecionar acento                                         3. colocar valor negativo na bomboniere</t>
+    <t>Validar preço de inteira para sessão em horário de matinê</t>
+  </si>
+  <si>
+    <t>O sistema está aberto na página principal e há sessão do filme 'Órbita Silenciosa' às 14:00.</t>
+  </si>
+  <si>
+    <t>1. Selecionar o filme 'Órbita Silenciosa'. 2. Escolher a sessão das 14:00 (2D). 3. Selecionar 1 assento. 4. Observar o valor do ingresso inteiro no resumo.</t>
+  </si>
+  <si>
+    <t>Filme: Órbita Silenciosa, Sessão: 14:00 (2D), Quantidade: 1 inteira.</t>
+  </si>
+  <si>
+    <t>O valor unitário do ingresso inteiro deve ser exibido como R$ 24,00.</t>
+  </si>
+  <si>
+    <t>CA01.3</t>
+  </si>
+  <si>
+    <t>Validar preço de inteira para sessão iniciada após as 17:00</t>
+  </si>
+  <si>
+    <t>O sistema está aberto na página principal.</t>
+  </si>
+  <si>
+    <t>1. Selecionar o filme 'O Último Farol'. 2. Escolher a sessão das 21:00 (2D). 3. Selecionar 1 assento. 4. Verificar o subtotal de ingressos.</t>
+  </si>
+  <si>
+    <t>Filme: O Último Farol, Sessão: 21:00 (2D), Quantidade: 1 inteira.</t>
+  </si>
+  <si>
+    <t>O valor unitário do ingresso inteiro deve ser de R$ 32,00.</t>
+  </si>
+  <si>
+    <t>CA02.2</t>
+  </si>
+  <si>
+    <t>Validar aplicação do adicional 3D para múltiplos ingressos</t>
+  </si>
+  <si>
+    <t>1. Selecionar o filme 'Órbita Silenciosa'. 2. Escolher a sessão das 20:30 (3D). 3. Selecionar 2 assentos. 4. Verificar o subtotal dos ingressos.</t>
+  </si>
+  <si>
+    <t>Filme: Órbita Silenciosa, Sessão: 20:30 (3D), Ingressos: 2 inteiras.</t>
+  </si>
+  <si>
+    <t>Cada ingresso deve custar R$ 32,00 + R$ 6,00 (totalizando R$ 38,00 cada), resultando em um subtotal de R$ 76,00.</t>
+  </si>
+  <si>
+    <t>CA03.2</t>
+  </si>
+  <si>
+    <t>Validar cálculo de meia-entrada em sessão 3D</t>
+  </si>
+  <si>
+    <t>1. Selecionar o filme 'Órbita Silenciosa'. 2. Escolher a sessão das 20:30 (3D). 3. Selecionar 1 assento. 4. Marcar o ingresso como meia-entrada. 5. Verificar o valor cobrado pelo ingresso.</t>
+  </si>
+  <si>
+    <t>Sessão: 20:30 (3D), Tipo de ingresso: 1 meia-entrada.</t>
+  </si>
+  <si>
+    <t>O valor da meia-entrada deve ser 50% do valor total do ingresso (R$ 38,00), resultando em R$ 19,00.</t>
+  </si>
+  <si>
+    <t>Verificar restrição de meia-entrada em sessão de pré-estreia</t>
+  </si>
+  <si>
+    <t>1. Selecionar o filme 'Cidade de Vidro' (Pré-estreia). 2. Escolher a sessão das 22:00 (2D). 3. Selecionar 1 assento. 4. Tentar marcar como meia-entrada. 5. Verificar o preço cobrado.</t>
+  </si>
+  <si>
+    <t>Sessão de pré-estreia, tentativa de seleção de meia-entrada.</t>
+  </si>
+  <si>
+    <t>A opção de meia-entrada não deve alterar o preço, cobrando o valor integral de R$ 32,00.</t>
+  </si>
+  <si>
+    <t>Validar limite máximo de 6 ingressos por pedido</t>
+  </si>
+  <si>
+    <t>O usuário selecionou uma sessão válida e já marcou 6 assentos no mapa da sala.</t>
+  </si>
+  <si>
+    <t>1. Clicar em um 7º assento livre no mapa da sala. 2. Observar o comportamento da interface.</t>
+  </si>
+  <si>
+    <t>Tentativa de seleção do 7º assento.</t>
+  </si>
+  <si>
+    <t>O sistema deve recusar a seleção do 7º assento e exibir um aviso ao cliente.</t>
+  </si>
+  <si>
+    <t>CA06.2</t>
+  </si>
+  <si>
+    <t>Desfazer seleção de assento ao clicar novamente</t>
+  </si>
+  <si>
+    <t>O usuário escolheu uma sessão e marcou 1 assento.</t>
+  </si>
+  <si>
+    <t>1. Clicar novamente sobre o assento já selecionado. 2. Verificar o status do assento e o valor do pedido.</t>
+  </si>
+  <si>
+    <t>Clique duplo no mesmo assento selecionado.</t>
+  </si>
+  <si>
+    <t>O assento deve ser liberado (desmarcado), retirado do mapa de seleção e o valor dos ingressos deve voltar a zero.</t>
+  </si>
+  <si>
+    <t>Validar quantidade máxima de itens na bomboniere</t>
+  </si>
+  <si>
+    <t>O usuário está na etapa de seleção da bomboniere.</t>
+  </si>
+  <si>
+    <t>1. Digitar o valor 12 no campo de quantidade da 'Pipoca pequena'. 2. Sair do campo (perder o foco). 3. Verificar o valor assumido pelo campo.</t>
+  </si>
+  <si>
+    <t>Quantidade informada: 12.</t>
+  </si>
+  <si>
+    <t>O sistema deve corrigir automaticamente o valor para o limite máximo permitido, que é 10.</t>
+  </si>
+  <si>
+    <t>CA08.2</t>
+  </si>
+  <si>
+    <t>Validar incidência da taxa de conveniência apenas sobre ingressos</t>
+  </si>
+  <si>
+    <t>O usuário adicionou 1 ingresso e 2 unidades de pipoca pequena ao pedido.</t>
+  </si>
+  <si>
+    <t>1. Visualizar o detalhamento do resumo de valores. 2. Calcular a taxa de conveniência aplicada.</t>
+  </si>
+  <si>
+    <t>1 Ingresso e 2 Pipocas pequenas.</t>
+  </si>
+  <si>
+    <t>A taxa de conveniência deve ser cobrada apenas com base na quantidade de ingressos (1 ingresso = R$ 2,50), sem incidir sobre os itens da bomboniere.</t>
+  </si>
+  <si>
+    <t>CA09.2</t>
+  </si>
+  <si>
+    <t>Tabela de Decisão</t>
+  </si>
+  <si>
+    <t>Validar flexibilidade de formatação no cupom CINE10</t>
+  </si>
+  <si>
+    <t>O usuário possui itens de ingresso no carrinho.</t>
+  </si>
+  <si>
+    <t>1. Digitar o cupom com espaços e letras minúsculas (` cIne10 `) no campo de cupons. 2. Aplicar o cupom. 3. Verificar se o desconto foi concedido.</t>
+  </si>
+  <si>
+    <t>String de cupom: ` cIne10 `</t>
+  </si>
+  <si>
+    <t>O cupom deve ser aceito independentemente de letras maiúsculas/minúsculas e espaços nas pontas, aplicando 10% de desconto sobre o subtotal de ingressos.</t>
+  </si>
+  <si>
+    <t>CA10.2</t>
+  </si>
+  <si>
+    <t>Validar rejeição do cupom PIPOCA5 abaixo do valor mínimo</t>
+  </si>
+  <si>
+    <t>O usuário possui itens de bomboniere com subtotal inferior a R$ 25,00 no carrinho (ex: 1 Refrigerante de R$ 9,50).</t>
+  </si>
+  <si>
+    <t>1. Inserir o cupom `PIPOCA5`. 2. Tentar aplicar. 3. Verificar a mensagem exibida.</t>
+  </si>
+  <si>
+    <t>Cupom: `PIPOCA5`, Subtotal da bomboniere: R$ 9,50.</t>
+  </si>
+  <si>
+    <t>O cupom deve ser recusado e uma mensagem explicativa de restrição deve ser exibida.</t>
+  </si>
+  <si>
+    <t>CA11.2</t>
+  </si>
+  <si>
+    <t>Validar remoção do desconto Pix ao alterar forma de pagamento</t>
+  </si>
+  <si>
+    <t>O usuário selecionou a forma de pagamento Pix e o desconto de 5% foi aplicado ao total.</t>
+  </si>
+  <si>
+    <t>1. Alterar a forma de pagamento de Pix para Cartão de Crédito. 2. Verificar o valor total do pedido.</t>
+  </si>
+  <si>
+    <t>Troca de Pix para Cartão.</t>
+  </si>
+  <si>
+    <t>O desconto de 5% associado ao Pix deve ser removido imediatamente do valor total.</t>
+  </si>
+  <si>
+    <t>CA12.1</t>
+  </si>
+  <si>
+    <t>Validar limite de parcelamento para pedidos abaixo de R$ 150,00</t>
+  </si>
+  <si>
+    <t>O usuário selecionou Cartão de Crédito como forma de pagamento e o valor total do pedido é de R$ 149,99.</t>
+  </si>
+  <si>
+    <t>1. Abrir o seletor de parcelas do cartão de crédito. 2. Verificar o número máximo de parcelas disponíveis.</t>
+  </si>
+  <si>
+    <t>Valor total do pedido: R$ 149,99.</t>
+  </si>
+  <si>
+    <t>O sistema deve permitir o parcelamento em no máximo 3x sem juros.</t>
+  </si>
+  <si>
+    <t>CA13.1</t>
+  </si>
+  <si>
+    <t>Validar validação de tamanho mínimo para o campo Nome Completo</t>
+  </si>
+  <si>
+    <t>O usuário chegou na etapa de preenchimento dos dados do comprador.</t>
+  </si>
+  <si>
+    <t>1. Digitar um nome com 2 caracteres ('An'). 2. Tentar prosseguir/confirmar a compra. 3. Limpar e digitar um nome com 3 caracteres ('Ana'). 4. Tentar prosseguir.</t>
+  </si>
+  <si>
+    <t>'An' (inválido) e 'Ana' (válido).</t>
+  </si>
+  <si>
+    <t>O nome com 2 caracteres deve ser recusado com mensagem de erro; o nome com 3 caracteres deve ser aceito.</t>
+  </si>
+  <si>
+    <t>Validar validação do formato do e-mail do comprador</t>
+  </si>
+  <si>
+    <t>O usuário está preenchendo os dados do comprador.</t>
+  </si>
+  <si>
+    <t>1. Informar um e-mail sem o caractere arroba (`clientecinema.com`). 2. Tentar confirmar a compra.</t>
+  </si>
+  <si>
+    <t>E-mail inválido: `clientecinema.com`</t>
+  </si>
+  <si>
+    <t>O sistema deve recusar o formato do e-mail, impedir a confirmação e exibir mensagem de erro correspondente.</t>
+  </si>
+  <si>
+    <t>CA16.1</t>
+  </si>
+  <si>
+    <t>Verificar persistência do pedido em andamento após recarregar a página (F5)</t>
+  </si>
+  <si>
+    <t>O usuário selecionou a sessão, assentos e alguns itens de bomboniere.</t>
+  </si>
+  <si>
+    <t>1. Pressionar a tecla `F5` para recarregar a página do navegador antes de confirmar a compra. 2. Verificar se os dados selecionados foram mantidos.</t>
+  </si>
+  <si>
+    <t>Ação de recarregar a página (F5).</t>
+  </si>
+  <si>
+    <t>A sessão, os assentos escolhidos e os itens da bomboniere devem continuar selecionados na interface após o refresh.</t>
+  </si>
+  <si>
+    <t>CA18.1</t>
+  </si>
+  <si>
+    <t>Validar proteção contra execução de tags HTML nos dados do comprador</t>
+  </si>
+  <si>
+    <t>O usuário está na tela de preenchimento dos dados do comprador.</t>
+  </si>
+  <si>
+    <t>1. Inserir tag HTML no campo de Nome Completo (`&lt;b&gt;Ana&lt;/b&gt;`). 2. Concluir a compra e verificar a tela de confirmação.</t>
+  </si>
+  <si>
+    <t>Nome: `&lt;b&gt;Ana&lt;/b&gt;`</t>
+  </si>
+  <si>
+    <t>O conteúdo deve ser exibido estritamente como texto literal (sem aplicação de formatação de negrito ou execução de script).</t>
+  </si>
+  <si>
+    <t>CA19.1</t>
+  </si>
+  <si>
+    <t>Validar navegação e fluxo de compra completo utilizando apenas o teclado</t>
+  </si>
+  <si>
+    <t>O sistema está aberto na página inicial, sem o uso do mouse.</t>
+  </si>
+  <si>
+    <t>1. Utilizar as teclas `Tab`, `Shift+Tab`, setas direcionais, `Enter` e `Espaço`. 2. Selecionar filme, sessão, assentos, preencher dados e confirmar a compra.</t>
+  </si>
+  <si>
+    <t>Comandos exclusivos via teclado.</t>
+  </si>
+  <si>
+    <t>Toda a jornada de compra deve ser concluída com sucesso sem a necessidade de interagir com o mouse.</t>
+  </si>
+  <si>
+    <t>CA20.1</t>
+  </si>
+  <si>
+    <t>Validar formatação padrão brasileira de moeda em todos os campos de valores</t>
+  </si>
+  <si>
+    <t>O usuário adicionou ingressos e itens ao carrinho.</t>
+  </si>
+  <si>
+    <t>1. Inspecionar todas as linhas de resumo de preços (ingressos, taxa, bomboniere, descontos e total).</t>
+  </si>
+  <si>
+    <t>Valores calculados no carrinho.</t>
+  </si>
+  <si>
+    <t>Todos os valores monetários devem seguir rigorosamente o padrão brasileiro com o prefixo 'R$', vírgula como separador decimal e duas casas decimais (ex: R$ 23,70).</t>
+  </si>
+  <si>
+    <t>CA21.1</t>
+  </si>
+  <si>
+    <t>Caixa Branca</t>
+  </si>
+  <si>
+    <t>Validar integridade dos preços contra manipulação via DevTools</t>
+  </si>
+  <si>
+    <t>O usuário está na etapa final de pagamento com produtos no carrinho.</t>
+  </si>
+  <si>
+    <t>1. Abrir as Ferramentas de Desenvolvedor (DevTools) do navegador. 2. Alterar o atributo de preço de um ingresso ou o valor total exibido no DOM. 3. Clicar em 'Confirmar compra' e verificar o valor registrado.</t>
+  </si>
+  <si>
+    <t>Manipulação manual de elementos HTML/atributos de preço via DevTools.</t>
+  </si>
+  <si>
+    <t>A alteração feita no cliente via DevTools não deve impactar o valor cobrado/processado pelo sistema de regras de negócio (backend simulado).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1833,6 +2067,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1906,7 +2146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -1961,6 +2201,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2999,7 +3242,7 @@
       </c>
       <c r="B5" s="18">
         <f>COUNTA('5_Casos_de_Teste'!G6:G45)</f>
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -3053,7 +3296,7 @@
       </c>
       <c r="B11" s="18">
         <f>COUNTIF('5_Casos_de_Teste'!D6:D45,"Valor limite")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -4765,7 +5008,7 @@
       <c r="N5" s="14"/>
       <c r="O5" s="14"/>
     </row>
-    <row r="6" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>171</v>
       </c>
@@ -4776,185 +5019,191 @@
         <v>512</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>463</v>
+        <v>162</v>
       </c>
       <c r="E6" s="8" t="s">
         <v>134</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>445</v>
+        <v>163</v>
       </c>
       <c r="G6" s="23" t="s">
+        <v>528</v>
+      </c>
+      <c r="H6" s="23" t="s">
         <v>529</v>
       </c>
-      <c r="H6" s="23" t="s">
+      <c r="I6" s="23" t="s">
         <v>530</v>
       </c>
-      <c r="I6" s="23" t="s">
-        <v>534</v>
-      </c>
-      <c r="J6" s="8"/>
+      <c r="J6" s="8" t="s">
+        <v>531</v>
+      </c>
       <c r="K6" s="23" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="L6" s="8"/>
       <c r="M6" s="8"/>
       <c r="N6" s="8"/>
       <c r="O6" s="8"/>
     </row>
-    <row r="7" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>172</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>443</v>
+        <v>433</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>525</v>
+        <v>533</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>463</v>
+        <v>444</v>
       </c>
       <c r="E7" s="8" t="s">
         <v>134</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>445</v>
+        <v>163</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>535</v>
-      </c>
-      <c r="J7" s="8"/>
+        <v>536</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>537</v>
+      </c>
       <c r="K7" s="23" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
       <c r="O7" s="8"/>
     </row>
-    <row r="8" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>173</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>454</v>
+        <v>443</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>526</v>
+        <v>539</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>463</v>
+        <v>162</v>
       </c>
       <c r="E8" s="8" t="s">
         <v>134</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>445</v>
+        <v>163</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="K8" s="23" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="8"/>
       <c r="O8" s="8"/>
     </row>
-    <row r="9" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="66" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>174</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>462</v>
+        <v>454</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>527</v>
+        <v>544</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="E9" s="8" t="s">
         <v>134</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>445</v>
+        <v>163</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>539</v>
+        <v>547</v>
       </c>
       <c r="K9" s="22" t="s">
-        <v>543</v>
+        <v>548</v>
       </c>
       <c r="L9" s="8"/>
       <c r="M9" s="8"/>
       <c r="N9" s="8"/>
       <c r="O9" s="8"/>
     </row>
-    <row r="10" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="66" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>175</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>134</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>445</v>
+        <v>163</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="H10" s="23" t="s">
-        <v>545</v>
+        <v>535</v>
       </c>
       <c r="I10" s="23" t="s">
-        <v>546</v>
-      </c>
-      <c r="J10" s="8"/>
+        <v>550</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>551</v>
+      </c>
       <c r="K10" s="23" t="s">
-        <v>547</v>
+        <v>552</v>
       </c>
       <c r="L10" s="8"/>
       <c r="M10" s="8"/>
       <c r="N10" s="8"/>
       <c r="O10" s="8"/>
     </row>
-    <row r="11" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>176</v>
       </c>
@@ -4962,71 +5211,77 @@
         <v>469</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>548</v>
+        <v>526</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>137</v>
+        <v>444</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>134</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>445</v>
+        <v>163</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>545</v>
+        <v>554</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>550</v>
-      </c>
-      <c r="J11" s="8"/>
+        <v>555</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>556</v>
+      </c>
       <c r="K11" s="23" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="L11" s="8"/>
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
       <c r="O11" s="8"/>
     </row>
-    <row r="12" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>177</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>134</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>445</v>
+        <v>163</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>553</v>
-      </c>
-      <c r="H12" s="8"/>
+        <v>559</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>560</v>
+      </c>
       <c r="I12" s="8" t="s">
-        <v>554</v>
-      </c>
-      <c r="J12" s="8"/>
+        <v>561</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>562</v>
+      </c>
       <c r="K12" s="8" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
       <c r="L12" s="8"/>
       <c r="M12" s="8"/>
       <c r="N12" s="8"/>
       <c r="O12" s="8"/>
     </row>
-    <row r="13" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>178</v>
       </c>
@@ -5034,7 +5289,7 @@
         <v>476</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>556</v>
+        <v>527</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>444</v>
@@ -5043,35 +5298,37 @@
         <v>134</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>434</v>
+        <v>163</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>557</v>
+        <v>564</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>558</v>
+        <v>565</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>559</v>
-      </c>
-      <c r="J13" s="8"/>
+        <v>566</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>567</v>
+      </c>
       <c r="K13" s="22" t="s">
-        <v>560</v>
+        <v>568</v>
       </c>
       <c r="L13" s="8"/>
       <c r="M13" s="8"/>
       <c r="N13" s="8"/>
       <c r="O13" s="8"/>
     </row>
-    <row r="14" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="66" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>179</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>561</v>
+        <v>569</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>162</v>
@@ -5080,226 +5337,452 @@
         <v>134</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>434</v>
+        <v>163</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>562</v>
-      </c>
-      <c r="H14" s="8"/>
+        <v>570</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>571</v>
+      </c>
       <c r="I14" s="23" t="s">
-        <v>563</v>
-      </c>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
+        <v>572</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>573</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>574</v>
+      </c>
       <c r="L14" s="22"/>
       <c r="M14" s="8"/>
       <c r="N14" s="8"/>
       <c r="O14" s="8"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="8"/>
+      <c r="B15" s="8" t="s">
+        <v>482</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>575</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>576</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>577</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>578</v>
+      </c>
+      <c r="I15" s="8" t="s">
+        <v>579</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>580</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>581</v>
+      </c>
       <c r="L15" s="8"/>
       <c r="M15" s="8"/>
       <c r="N15" s="8"/>
       <c r="O15" s="8"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
+      <c r="B16" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>582</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>444</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>583</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>584</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>585</v>
+      </c>
+      <c r="J16" s="8" t="s">
+        <v>586</v>
+      </c>
+      <c r="K16" s="8" t="s">
+        <v>587</v>
+      </c>
       <c r="L16" s="8"/>
       <c r="M16" s="8"/>
       <c r="N16" s="8"/>
       <c r="O16" s="8"/>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
+    <row r="17" spans="1:15" s="25" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="28" t="s">
         <v>182</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
-      <c r="M17" s="8"/>
-      <c r="N17" s="8"/>
-      <c r="O17" s="8"/>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="B17" s="23" t="s">
+        <v>484</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>588</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="E17" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="G17" s="23" t="s">
+        <v>589</v>
+      </c>
+      <c r="H17" s="23" t="s">
+        <v>590</v>
+      </c>
+      <c r="I17" s="23" t="s">
+        <v>591</v>
+      </c>
+      <c r="J17" s="23" t="s">
+        <v>592</v>
+      </c>
+      <c r="K17" s="23" t="s">
+        <v>593</v>
+      </c>
+      <c r="L17" s="23"/>
+      <c r="M17" s="23"/>
+      <c r="N17" s="23"/>
+      <c r="O17" s="23"/>
+    </row>
+    <row r="18" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
+      <c r="B18" s="8" t="s">
+        <v>486</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>594</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>444</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>595</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>596</v>
+      </c>
+      <c r="I18" s="8" t="s">
+        <v>597</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>598</v>
+      </c>
+      <c r="K18" s="8" t="s">
+        <v>599</v>
+      </c>
       <c r="L18" s="8"/>
       <c r="M18" s="8"/>
       <c r="N18" s="8"/>
       <c r="O18" s="8"/>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
+      <c r="B19" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>600</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>444</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>601</v>
+      </c>
+      <c r="H19" s="8" t="s">
+        <v>602</v>
+      </c>
+      <c r="I19" s="8" t="s">
+        <v>603</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>604</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>605</v>
+      </c>
       <c r="L19" s="8"/>
       <c r="M19" s="8"/>
       <c r="N19" s="8"/>
       <c r="O19" s="8"/>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
+      <c r="B20" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>606</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>607</v>
+      </c>
+      <c r="I20" s="8" t="s">
+        <v>608</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>609</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>610</v>
+      </c>
       <c r="L20" s="8"/>
       <c r="M20" s="8"/>
       <c r="N20" s="8"/>
       <c r="O20" s="8"/>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
-      <c r="K21" s="8"/>
+      <c r="B21" s="8" t="s">
+        <v>490</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>611</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>612</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>613</v>
+      </c>
+      <c r="I21" s="8" t="s">
+        <v>614</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>615</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>616</v>
+      </c>
       <c r="L21" s="8"/>
       <c r="M21" s="8"/>
       <c r="N21" s="8"/>
       <c r="O21" s="8"/>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8"/>
+      <c r="B22" s="8" t="s">
+        <v>491</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>617</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>618</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>619</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>620</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>621</v>
+      </c>
+      <c r="K22" s="8" t="s">
+        <v>622</v>
+      </c>
       <c r="L22" s="8"/>
       <c r="M22" s="8"/>
       <c r="N22" s="8"/>
       <c r="O22" s="8"/>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
-      <c r="K23" s="8"/>
+      <c r="B23" s="8" t="s">
+        <v>492</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>623</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>625</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>626</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>627</v>
+      </c>
+      <c r="K23" s="8" t="s">
+        <v>628</v>
+      </c>
       <c r="L23" s="8"/>
       <c r="M23" s="8"/>
       <c r="N23" s="8"/>
       <c r="O23" s="8"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" ht="66" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="8"/>
-      <c r="K24" s="8"/>
+      <c r="B24" s="8" t="s">
+        <v>493</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>629</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>630</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>631</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>632</v>
+      </c>
+      <c r="J24" s="8" t="s">
+        <v>633</v>
+      </c>
+      <c r="K24" s="8" t="s">
+        <v>634</v>
+      </c>
       <c r="L24" s="8"/>
       <c r="M24" s="8"/>
       <c r="N24" s="8"/>
       <c r="O24" s="8"/>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" ht="66" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
-      <c r="K25" s="8"/>
+      <c r="B25" s="8" t="s">
+        <v>494</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>635</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>636</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>637</v>
+      </c>
+      <c r="H25" s="8" t="s">
+        <v>638</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>639</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>640</v>
+      </c>
+      <c r="K25" s="8" t="s">
+        <v>641</v>
+      </c>
       <c r="L25" s="8"/>
       <c r="M25" s="8"/>
       <c r="N25" s="8"/>

</xml_diff>